<commit_message>
Import documents completed with correct reference logic
</commit_message>
<xml_diff>
--- a/Files/Madden26/IE/Season2/FreeAgency/Input/Team.xlsx
+++ b/Files/Madden26/IE/Season2/FreeAgency/Input/Team.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenTools/Files/Madden26/IE/Season2/FreeAgency/Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="115" documentId="11_0CC34E5D2364FF18F55B1250EA3161BA9358D94E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7281C9FA-6C83-4C82-A4F8-4F0397B32E20}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="11_0CC34E5D2364FF18F55B1250EA3161BA9358D94E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F255EE05-B057-408B-ABB2-EEE3F0592B0C}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -8032,10 +8032,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8361,18 +8357,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:KU33"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.25" customWidth="1"/>
-    <col min="5" max="5" width="11.75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.75" customWidth="1"/>
-    <col min="7" max="7" width="16.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.19921875" customWidth="1"/>
+    <col min="5" max="5" width="11.69921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.69921875" customWidth="1"/>
+    <col min="7" max="7" width="16.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2644</v>
       </c>
@@ -9295,7 +9291,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="2" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>377</v>
       </c>
@@ -9307,7 +9303,7 @@
         <v>11</v>
       </c>
       <c r="D2">
-        <v>-3112</v>
+        <v>854</v>
       </c>
       <c r="E2">
         <v>14</v>
@@ -10219,7 +10215,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>463</v>
       </c>
@@ -10231,7 +10227,7 @@
         <v>8</v>
       </c>
       <c r="D3">
-        <v>3629</v>
+        <v>5629</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -11143,7 +11139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>543</v>
       </c>
@@ -11155,7 +11151,7 @@
         <v>10</v>
       </c>
       <c r="D4">
-        <v>1818</v>
+        <v>3818</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -12067,7 +12063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>615</v>
       </c>
@@ -12079,7 +12075,7 @@
         <v>9</v>
       </c>
       <c r="D5">
-        <v>5341</v>
+        <v>7341</v>
       </c>
       <c r="E5">
         <v>2</v>
@@ -12991,7 +12987,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>692</v>
       </c>
@@ -13003,7 +12999,7 @@
         <v>8</v>
       </c>
       <c r="D6">
-        <v>-3231</v>
+        <v>478</v>
       </c>
       <c r="E6">
         <v>3</v>
@@ -13915,7 +13911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>769</v>
       </c>
@@ -14839,7 +14835,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>844</v>
       </c>
@@ -14851,7 +14847,7 @@
         <v>5</v>
       </c>
       <c r="D8">
-        <v>1925</v>
+        <v>3925</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -15763,7 +15759,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>917</v>
       </c>
@@ -15775,7 +15771,7 @@
         <v>8</v>
       </c>
       <c r="D9">
-        <v>8845</v>
+        <v>10845</v>
       </c>
       <c r="E9">
         <v>6</v>
@@ -16687,7 +16683,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>989</v>
       </c>
@@ -16699,7 +16695,7 @@
         <v>13</v>
       </c>
       <c r="D10">
-        <v>-730</v>
+        <v>1270</v>
       </c>
       <c r="E10">
         <v>7</v>
@@ -17611,7 +17607,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>1068</v>
       </c>
@@ -17623,7 +17619,7 @@
         <v>11</v>
       </c>
       <c r="D11">
-        <v>3507</v>
+        <v>5507</v>
       </c>
       <c r="E11">
         <v>8</v>
@@ -18535,7 +18531,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>1143</v>
       </c>
@@ -18547,7 +18543,7 @@
         <v>5</v>
       </c>
       <c r="D12">
-        <v>3931</v>
+        <v>5931</v>
       </c>
       <c r="E12">
         <v>9</v>
@@ -19459,7 +19455,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>1216</v>
       </c>
@@ -19471,7 +19467,7 @@
         <v>12</v>
       </c>
       <c r="D13">
-        <v>1100</v>
+        <v>3100</v>
       </c>
       <c r="E13">
         <v>25</v>
@@ -20383,7 +20379,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>1290</v>
       </c>
@@ -20395,7 +20391,7 @@
         <v>10</v>
       </c>
       <c r="D14">
-        <v>-6343</v>
+        <v>167</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -21307,7 +21303,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>1363</v>
       </c>
@@ -21319,7 +21315,7 @@
         <v>8</v>
       </c>
       <c r="D15">
-        <v>4488</v>
+        <v>6488</v>
       </c>
       <c r="E15">
         <v>11</v>
@@ -22231,7 +22227,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>1433</v>
       </c>
@@ -22243,7 +22239,7 @@
         <v>4</v>
       </c>
       <c r="D16">
-        <v>-6992</v>
+        <v>267</v>
       </c>
       <c r="E16">
         <v>12</v>
@@ -23155,7 +23151,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>1506</v>
       </c>
@@ -23167,7 +23163,7 @@
         <v>7</v>
       </c>
       <c r="D17">
-        <v>5594</v>
+        <v>7594</v>
       </c>
       <c r="E17">
         <v>13</v>
@@ -24079,7 +24075,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>1576</v>
       </c>
@@ -24091,7 +24087,7 @@
         <v>11</v>
       </c>
       <c r="D18">
-        <v>2447</v>
+        <v>4447</v>
       </c>
       <c r="E18">
         <v>15</v>
@@ -25003,7 +24999,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>1649</v>
       </c>
@@ -25015,7 +25011,7 @@
         <v>11</v>
       </c>
       <c r="D19">
-        <v>-366</v>
+        <v>1634</v>
       </c>
       <c r="E19">
         <v>16</v>
@@ -25927,7 +25923,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>1718</v>
       </c>
@@ -25939,7 +25935,7 @@
         <v>5</v>
       </c>
       <c r="D20">
-        <v>12401</v>
+        <v>12404</v>
       </c>
       <c r="E20">
         <v>17</v>
@@ -26851,7 +26847,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>1791</v>
       </c>
@@ -26863,7 +26859,7 @@
         <v>9</v>
       </c>
       <c r="D21">
-        <v>3070</v>
+        <v>5070</v>
       </c>
       <c r="E21">
         <v>18</v>
@@ -27775,7 +27771,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>1865</v>
       </c>
@@ -27787,7 +27783,7 @@
         <v>14</v>
       </c>
       <c r="D22">
-        <v>-3474</v>
+        <v>690</v>
       </c>
       <c r="E22">
         <v>19</v>
@@ -28699,7 +28695,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>1935</v>
       </c>
@@ -28711,7 +28707,7 @@
         <v>6</v>
       </c>
       <c r="D23">
-        <v>5251</v>
+        <v>7251</v>
       </c>
       <c r="E23">
         <v>20</v>
@@ -29623,7 +29619,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>2002</v>
       </c>
@@ -29635,7 +29631,7 @@
         <v>10</v>
       </c>
       <c r="D24">
-        <v>354</v>
+        <v>2354</v>
       </c>
       <c r="E24">
         <v>21</v>
@@ -30547,7 +30543,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>2074</v>
       </c>
@@ -30559,7 +30555,7 @@
         <v>10</v>
       </c>
       <c r="D25">
-        <v>4020</v>
+        <v>6020</v>
       </c>
       <c r="E25">
         <v>22</v>
@@ -31471,7 +31467,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>2145</v>
       </c>
@@ -31483,7 +31479,7 @@
         <v>7</v>
       </c>
       <c r="D26">
-        <v>3978</v>
+        <v>5978</v>
       </c>
       <c r="E26">
         <v>23</v>
@@ -32395,7 +32391,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>2216</v>
       </c>
@@ -32407,7 +32403,7 @@
         <v>6</v>
       </c>
       <c r="D27">
-        <v>1500</v>
+        <v>3500</v>
       </c>
       <c r="E27">
         <v>24</v>
@@ -33319,7 +33315,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2286</v>
       </c>
@@ -34243,7 +34239,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>2355</v>
       </c>
@@ -34255,7 +34251,7 @@
         <v>10</v>
       </c>
       <c r="D29">
-        <v>4888</v>
+        <v>6888</v>
       </c>
       <c r="E29">
         <v>27</v>
@@ -35167,7 +35163,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>2426</v>
       </c>
@@ -35179,7 +35175,7 @@
         <v>4</v>
       </c>
       <c r="D30">
-        <v>5694</v>
+        <v>7694</v>
       </c>
       <c r="E30">
         <v>28</v>
@@ -36091,7 +36087,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>1065</v>
       </c>
@@ -36103,7 +36099,7 @@
         <v>12</v>
       </c>
       <c r="D31">
-        <v>2759</v>
+        <v>4759</v>
       </c>
       <c r="E31">
         <v>31</v>
@@ -37015,7 +37011,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>2568</v>
       </c>
@@ -37027,7 +37023,7 @@
         <v>9</v>
       </c>
       <c r="D32">
-        <v>-2344</v>
+        <v>750</v>
       </c>
       <c r="E32">
         <v>29</v>
@@ -37939,7 +37935,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:307" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:307" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>2640</v>
       </c>
@@ -37951,7 +37947,7 @@
         <v>8</v>
       </c>
       <c r="D33">
-        <v>2881</v>
+        <v>4881</v>
       </c>
       <c r="E33">
         <v>30</v>

</xml_diff>